<commit_message>
Add team groups and settled-match lockout
</commit_message>
<xml_diff>
--- a/world_cup_cash_google_sheets_template_v1.xlsx
+++ b/world_cup_cash_google_sheets_template_v1.xlsx
@@ -701,11 +701,6 @@
           <t>setup</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -726,11 +721,6 @@
           <t>future</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -751,11 +741,6 @@
           <t>future</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -776,11 +761,6 @@
           <t>future</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -801,11 +781,6 @@
           <t>future</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -826,11 +801,6 @@
           <t>future</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -851,11 +821,6 @@
           <t>future</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -876,11 +841,6 @@
           <t>future</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -901,11 +861,6 @@
           <t>future</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -921,7 +876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -930,7 +885,7 @@
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="38" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
   </cols>
@@ -966,17 +921,22 @@
           <t>team_slug</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>flag_image</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>emblem_image</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>star_player_image</t>
         </is>
@@ -1015,15 +975,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>flags/algeria-flag.png</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>emblems/algeria-emblem.png</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>players/algeria-player.png</t>
         </is>
@@ -1062,15 +1027,20 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>flags/argentina-flag.png</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>emblems/argentina-emblem.png</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>players/argentina-player.png</t>
         </is>
@@ -1109,15 +1079,20 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>flags/australia-flag.png</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>emblems/australia-emblem.png</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>players/australia-player.png</t>
         </is>
@@ -1156,15 +1131,20 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>flags/austria-flag.png</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>emblems/austria-emblem.png</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>players/austria-player.png</t>
         </is>
@@ -1203,15 +1183,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>flags/belgium-flag.png</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>emblems/belgium-emblem.png</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>players/belgium-player.png</t>
         </is>
@@ -1250,15 +1235,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>flags/bosnia-herzegovina-flag.png</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>emblems/bosnia-herzegovina-emblem.png</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>players/bosnia-herzegovina-player.png</t>
         </is>
@@ -1297,15 +1287,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>flags/brazil-flag.png</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>emblems/brazil-emblem.png</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>players/brazil-player.png</t>
         </is>
@@ -1344,15 +1339,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>flags/cote-divoire-flag.png</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>emblems/cote-divoire-emblem.png</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>players/cote-divoire-player.png</t>
         </is>
@@ -1391,15 +1391,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>flags/canada-flag.png</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>emblems/canada-emblem.png</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>players/canada-player.png</t>
         </is>
@@ -1438,15 +1443,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>flags/cape-verde-flag.png</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>emblems/cape-verde-emblem.png</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>players/cape-verde-player.png</t>
         </is>
@@ -1485,15 +1495,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>flags/colombia-flag.png</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>emblems/colombia-emblem.png</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>players/colombia-player.png</t>
         </is>
@@ -1532,15 +1547,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>flags/croatia-flag.png</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>emblems/croatia-emblem.png</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>players/croatia-player.png</t>
         </is>
@@ -1579,15 +1599,20 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>flags/curacao-flag.png</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>emblems/curacao-emblem.png</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>players/curacao-player.png</t>
         </is>
@@ -1626,15 +1651,20 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>flags/czechia-flag.png</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>emblems/czechia-emblem.png</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>players/czechia-player.png</t>
         </is>
@@ -1673,15 +1703,20 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>flags/dr-congo-flag.png</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>emblems/dr-congo-emblem.png</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>players/dr-congo-player.png</t>
         </is>
@@ -1720,15 +1755,20 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>flags/ecuador-flag.png</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>emblems/ecuador-emblem.png</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>players/ecuador-player.png</t>
         </is>
@@ -1767,15 +1807,20 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
           <t>flags/egypt-flag.png</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>emblems/egypt-emblem.png</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>players/egypt-player.png</t>
         </is>
@@ -1814,15 +1859,20 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
           <t>flags/england-flag.png</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>emblems/england-emblem.png</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>players/england-player.png</t>
         </is>
@@ -1861,15 +1911,20 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
           <t>flags/france-flag.png</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>emblems/france-emblem.png</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>players/france-player.png</t>
         </is>
@@ -1908,15 +1963,20 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
           <t>flags/germany-flag.png</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>emblems/germany-emblem.png</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>players/germany-player.png</t>
         </is>
@@ -1955,15 +2015,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
           <t>flags/ghana-flag.png</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>emblems/ghana-emblem.png</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>players/ghana-player.png</t>
         </is>
@@ -2002,15 +2067,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>flags/haiti-flag.png</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>emblems/haiti-emblem.png</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>players/haiti-player.png</t>
         </is>
@@ -2049,15 +2119,20 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
           <t>flags/iran-flag.png</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>emblems/iran-emblem.png</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>players/iran-player.png</t>
         </is>
@@ -2096,15 +2171,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
           <t>flags/iraq-flag.png</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>emblems/iraq-emblem.png</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>players/iraq-player.png</t>
         </is>
@@ -2143,15 +2223,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
           <t>flags/japan-flag.png</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>emblems/japan-emblem.png</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>players/japan-player.png</t>
         </is>
@@ -2190,15 +2275,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
           <t>flags/jordan-flag.png</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>emblems/jordan-emblem.png</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>players/jordan-player.png</t>
         </is>
@@ -2237,15 +2327,20 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
           <t>flags/mexico-flag.png</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>emblems/mexico-emblem.png</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>players/mexico-player.png</t>
         </is>
@@ -2284,15 +2379,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
           <t>flags/morocco-flag.png</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>emblems/morocco-emblem.png</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>players/morocco-player.png</t>
         </is>
@@ -2331,15 +2431,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
           <t>flags/netherlands-flag.png</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>emblems/netherlands-emblem.png</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>players/netherlands-player.png</t>
         </is>
@@ -2378,15 +2483,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
           <t>flags/new-zealand-flag.png</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>emblems/new-zealand-emblem.png</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>players/new-zealand-player.png</t>
         </is>
@@ -2425,15 +2535,20 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
           <t>flags/norway-flag.png</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>emblems/norway-emblem.png</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>players/norway-player.png</t>
         </is>
@@ -2472,15 +2587,20 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
           <t>flags/panama-flag.png</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>emblems/panama-emblem.png</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>players/panama-player.png</t>
         </is>
@@ -2519,15 +2639,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
           <t>flags/paraguay-flag.png</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>emblems/paraguay-emblem.png</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>players/paraguay-player.png</t>
         </is>
@@ -2566,15 +2691,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
           <t>flags/portugal-flag.png</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>emblems/portugal-emblem.png</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>players/portugal-player.png</t>
         </is>
@@ -2613,15 +2743,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
           <t>flags/qatar-flag.png</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>emblems/qatar-emblem.png</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>players/qatar-player.png</t>
         </is>
@@ -2660,15 +2795,20 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
           <t>flags/saudi-arabia-flag.png</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>emblems/saudi-arabia-emblem.png</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>players/saudi-arabia-player.png</t>
         </is>
@@ -2707,15 +2847,20 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
           <t>flags/scotland-flag.png</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>emblems/scotland-emblem.png</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>players/scotland-player.png</t>
         </is>
@@ -2754,15 +2899,20 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
           <t>flags/senegal-flag.png</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>emblems/senegal-emblem.png</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>players/senegal-player.png</t>
         </is>
@@ -2801,15 +2951,20 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
           <t>flags/south-africa-flag.png</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>emblems/south-africa-emblem.png</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>players/south-africa-player.png</t>
         </is>
@@ -2848,15 +3003,20 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
           <t>flags/south-korea-flag.png</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>emblems/south-korea-emblem.png</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>players/south-korea-player.png</t>
         </is>
@@ -2895,15 +3055,20 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
           <t>flags/spain-flag.png</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>emblems/spain-emblem.png</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>players/spain-player.png</t>
         </is>
@@ -2942,15 +3107,20 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
           <t>flags/sweden-flag.png</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>emblems/sweden-emblem.png</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>players/sweden-player.png</t>
         </is>
@@ -2989,15 +3159,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
           <t>flags/switzerland-flag.png</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>emblems/switzerland-emblem.png</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>players/switzerland-player.png</t>
         </is>
@@ -3036,15 +3211,20 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
           <t>flags/turkiye-flag.png</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>emblems/turkiye-emblem.png</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>players/turkiye-player.png</t>
         </is>
@@ -3083,15 +3263,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
           <t>flags/tunisia-flag.png</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>emblems/tunisia-emblem.png</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>players/tunisia-player.png</t>
         </is>
@@ -3130,15 +3315,20 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
           <t>flags/united-states-flag.png</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>emblems/united-states-emblem.png</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>players/united-states-player.png</t>
         </is>
@@ -3177,15 +3367,20 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
           <t>flags/uruguay-flag.png</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>emblems/uruguay-emblem.png</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>players/uruguay-player.png</t>
         </is>
@@ -3224,15 +3419,20 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
           <t>flags/uzbekistan-flag.png</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>emblems/uzbekistan-emblem.png</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t>players/uzbekistan-player.png</t>
         </is>
@@ -3372,9 +3572,6 @@
           <t>4.33</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>future</t>
@@ -3422,9 +3619,6 @@
           <t>3.2</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>future</t>
@@ -3472,9 +3666,6 @@
           <t>3.8</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>future</t>
@@ -3522,9 +3713,6 @@
           <t>3.55</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>future</t>
@@ -3572,9 +3760,6 @@
           <t>5.75</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>future</t>
@@ -3622,9 +3807,6 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>future</t>
@@ -3672,9 +3854,6 @@
           <t>4.9</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>future</t>
@@ -3722,9 +3901,6 @@
           <t>3.75</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>future</t>
@@ -3772,9 +3948,6 @@
           <t>19</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>future</t>
@@ -3822,9 +3995,6 @@
           <t>3.75</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>future</t>
@@ -3872,9 +4042,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
           <t>future</t>
@@ -3922,9 +4089,6 @@
           <t>3.45</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>future</t>
@@ -3972,9 +4136,6 @@
           <t>11</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>future</t>
@@ -4022,9 +4183,6 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>future</t>
@@ -4072,9 +4230,6 @@
           <t>4.4</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>future</t>
@@ -4122,9 +4277,6 @@
           <t>3.65</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>future</t>
@@ -4172,9 +4324,6 @@
           <t>4.5</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>future</t>
@@ -4222,9 +4371,6 @@
           <t>6.25</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>future</t>
@@ -4272,9 +4418,6 @@
           <t>4.75</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>future</t>
@@ -4322,9 +4465,6 @@
           <t>5.5</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>future</t>
@@ -4372,9 +4512,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>future</t>
@@ -4422,9 +4559,6 @@
           <t>3.85</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>future</t>
@@ -4472,9 +4606,6 @@
           <t>3.9</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>future</t>
@@ -4522,9 +4653,6 @@
           <t>4.5</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>future</t>
@@ -4567,10 +4695,6 @@
           <t>4</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>future</t>
@@ -4618,9 +4742,6 @@
           <t>4.2</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>future</t>
@@ -4668,9 +4789,6 @@
           <t>4.3</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>future</t>
@@ -4718,9 +4836,6 @@
           <t>3.7</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>future</t>
@@ -4763,10 +4878,6 @@
           <t>5</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>future</t>
@@ -4809,10 +4920,6 @@
           <t>2.1</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>future</t>
@@ -4855,10 +4962,6 @@
           <t>66</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>future</t>
@@ -4901,10 +5004,6 @@
           <t>3.4</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>future</t>
@@ -4947,10 +5046,6 @@
           <t>5.1</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>future</t>
@@ -4993,10 +5088,6 @@
           <t>5.7</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>future</t>
@@ -5039,10 +5130,6 @@
           <t>13</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>future</t>
@@ -5085,10 +5172,6 @@
           <t>1.87</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
           <t>future</t>
@@ -5131,10 +5214,6 @@
           <t>21</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
           <t>future</t>
@@ -5177,10 +5256,6 @@
           <t>8</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
           <t>future</t>
@@ -5223,10 +5298,6 @@
           <t>7.5</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
           <t>future</t>
@@ -5269,10 +5340,6 @@
           <t>1.71</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
           <t>future</t>
@@ -5315,10 +5382,6 @@
           <t>5.5</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
           <t>future</t>
@@ -5361,10 +5424,6 @@
           <t>21</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
           <t>future</t>
@@ -5407,10 +5466,6 @@
           <t>3.7</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
           <t>future</t>
@@ -5453,10 +5508,6 @@
           <t>1.71</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
           <t>future</t>
@@ -5499,10 +5550,6 @@
           <t>17</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
           <t>future</t>
@@ -5545,10 +5592,6 @@
           <t>9</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
           <t>future</t>
@@ -5591,10 +5634,6 @@
           <t>1.54</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
           <t>future</t>
@@ -5637,10 +5676,6 @@
           <t>7.5</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
           <t>future</t>
@@ -5673,12 +5708,6 @@
           <t>canada</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
           <t>future</t>
@@ -5711,12 +5740,6 @@
           <t>qatar</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
           <t>future</t>
@@ -5759,10 +5782,6 @@
           <t>8.5</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
           <t>future</t>
@@ -5795,12 +5814,6 @@
           <t>haiti</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
           <t>future</t>
@@ -5833,12 +5846,6 @@
           <t>czechia</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
           <t>future</t>
@@ -5871,12 +5878,6 @@
           <t>south-africa</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
           <t>future</t>
@@ -5909,12 +5910,6 @@
           <t>germany</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
           <t>future</t>
@@ -5947,12 +5942,6 @@
           <t>cote-divoire</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
           <t>future</t>
@@ -5985,12 +5974,6 @@
           <t>netherlands</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
           <t>future</t>
@@ -6023,12 +6006,6 @@
           <t>sweden</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
           <t>future</t>
@@ -6061,12 +6038,6 @@
           <t>turkiye</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
           <t>future</t>
@@ -6099,12 +6070,6 @@
           <t>australia</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
           <t>future</t>
@@ -6137,12 +6102,6 @@
           <t>france</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
           <t>future</t>
@@ -6175,12 +6134,6 @@
           <t>iraq</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
           <t>future</t>
@@ -6213,12 +6166,6 @@
           <t>spain</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
           <t>future</t>
@@ -6251,12 +6198,6 @@
           <t>saudi-arabia</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
           <t>future</t>
@@ -6289,12 +6230,6 @@
           <t>belgium</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
           <t>future</t>
@@ -6327,12 +6262,6 @@
           <t>iran</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
           <t>future</t>
@@ -6365,12 +6294,6 @@
           <t>england</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
           <t>future</t>
@@ -6403,12 +6326,6 @@
           <t>ghana</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
           <t>future</t>
@@ -6441,12 +6358,6 @@
           <t>portugal</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
           <t>future</t>
@@ -6479,12 +6390,6 @@
           <t>uzbekistan</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
           <t>future</t>
@@ -6517,12 +6422,6 @@
           <t>jordan</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
           <t>future</t>
@@ -6555,12 +6454,6 @@
           <t>austria</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
           <t>future</t>
@@ -6593,12 +6486,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
           <t>future</t>
@@ -6631,12 +6518,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
           <t>future</t>
@@ -6669,12 +6550,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
           <t>future</t>
@@ -6707,12 +6582,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
           <t>future</t>
@@ -6745,12 +6614,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
           <t>future</t>
@@ -6783,12 +6646,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
           <t>future</t>
@@ -6821,12 +6678,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
           <t>future</t>
@@ -6859,12 +6710,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
           <t>future</t>
@@ -6897,12 +6742,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
           <t>future</t>
@@ -6935,12 +6774,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
           <t>future</t>
@@ -6973,12 +6806,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
           <t>future</t>
@@ -7011,12 +6838,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr"/>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
           <t>future</t>
@@ -7049,12 +6870,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
           <t>future</t>
@@ -7087,12 +6902,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
           <t>future</t>
@@ -7125,12 +6934,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
           <t>future</t>
@@ -7163,12 +6966,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
           <t>future</t>
@@ -7201,12 +6998,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
           <t>future</t>
@@ -7239,12 +7030,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr"/>
-      <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr"/>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
           <t>future</t>
@@ -7277,12 +7062,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr"/>
-      <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
           <t>future</t>
@@ -7315,12 +7094,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
           <t>future</t>
@@ -7353,12 +7126,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr"/>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
           <t>future</t>
@@ -7391,12 +7158,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr"/>
-      <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr"/>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
           <t>future</t>
@@ -7429,12 +7190,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
           <t>future</t>
@@ -7467,12 +7222,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr"/>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
           <t>future</t>
@@ -7505,12 +7254,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
           <t>future</t>
@@ -7543,12 +7286,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
-      <c r="H99" t="inlineStr"/>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
           <t>future</t>
@@ -7581,12 +7318,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
           <t>future</t>
@@ -7619,12 +7350,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
           <t>future</t>
@@ -7657,12 +7382,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
           <t>future</t>
@@ -7695,12 +7414,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
-      <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
-      <c r="I103" t="inlineStr"/>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
           <t>future</t>
@@ -7733,12 +7446,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
           <t>future</t>
@@ -7771,12 +7478,6 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr"/>
-      <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
-      <c r="I105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
           <t>future</t>

</xml_diff>